<commit_message>
docs: add more verified QCNN literature
</commit_message>
<xml_diff>
--- a/metadata/QCNN.xlsx
+++ b/metadata/QCNN.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2d5cf8588ae64b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb9a6fd1006544948"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -625,19 +625,19 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
-        <x:v>Subspace preserving quantum convolutional neural network architectures</x:v>
+        <x:v>Quantum convolutional neural network for MRI brain tumor analysis: Binary and multiclass classification using a four-qubit architecture</x:v>
       </x:c>
       <x:c r="B6" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>IOP Publishing</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
-        <x:v>Léo Monbroussou; Jonas Landman; Letao Wang; Alex B. Grilo; Elham Kashefi</x:v>
+        <x:v>Sitti Yani; Sugih Pratama Nugraha; Ariiq Islam Alfajri; Tony Sumaryada; Duong Thanh Tai; Hiba Omer; Nissren Tamam; Abdelmoneim Sulieman</x:v>
       </x:c>
       <x:c r="E6" s="2" t="str">
-        <x:v>https://doi.org/10.1088/2058-9565/adbf43</x:v>
+        <x:v>https://doi.org/10.1016/j.radphyschem.2025.113545</x:v>
       </x:c>
       <x:c r="F6" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -645,19 +645,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="str">
-        <x:v>Computation-efficient quantum convolutional neural networks for autonomous driving applications</x:v>
+        <x:v>Quantum convolutional neural network-based hybrid network for remote sensing image classification</x:v>
       </x:c>
       <x:c r="B7" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>Springer Nature</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
-        <x:v>Emily Jimin Roh; Chaemoon Im; Wonjun Jeong; Soohyun Park</x:v>
+        <x:v>H. N. Mahendra; V. Pushpalatha; S. Mallikarjunaswamy; S. Rama Subramoniam; J. Praveen</x:v>
       </x:c>
       <x:c r="E7" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s11227-025-07507-0</x:v>
+        <x:v>https://doi.org/10.1016/j.engappai.2025.113195</x:v>
       </x:c>
       <x:c r="F7" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -665,19 +665,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str">
-        <x:v>A multi-topology quantum convolutional neural network with qubit-measurement attention for image classification</x:v>
+        <x:v>A novel qVGG-4 model for optimizing a parameterized quantum circuit in a quantum-IoT-based brain tumor detection and monitoring system</x:v>
       </x:c>
       <x:c r="B8" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
         <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>QingShan Wu; WenJie Liu; XinRan Li; Zhaofeng Su; Jian Lei</x:v>
+        <x:v>Md Taimur Ahad; Bo Song; Yan Li</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.engappai.2025.111705</x:v>
+        <x:v>https://doi.org/10.1016/j.cmpb.2026.109362</x:v>
       </x:c>
       <x:c r="F8" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -685,19 +685,19 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>Quantum convolutional neural network based on variational quantum circuits.</x:v>
+        <x:v>A novel quantum convolutional neural network framework for quantum-enhanced classification of pixelated colour images</x:v>
       </x:c>
       <x:c r="B9" s="2" t="n">
-        <x:v>2024</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>Optics Communications</x:v>
+        <x:v>Nature Portfolio</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>Gong, Li-Hua, et al.</x:v>
+        <x:v>Chisomo Daka; Somnath Bhattacharyya</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0030401823007411</x:v>
+        <x:v>https://doi.org/10.1038/s41598-026-45140-w</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -705,19 +705,19 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
-        <x:v>Quantum Convolutional Neural Networks are (Effectively) Classically Simulable</x:v>
+        <x:v>Subspace preserving quantum convolutional neural network architectures</x:v>
       </x:c>
       <x:c r="B10" s="2" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>IOP Publishing</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
-        <x:v>Bermejo, Pablo, et al.</x:v>
+        <x:v>Léo Monbroussou; Jonas Landman; Letao Wang; Alex B. Grilo; Elham Kashefi</x:v>
       </x:c>
       <x:c r="E10" s="2" t="str">
-        <x:v>https://arxiv.org/pdf/2408.12739</x:v>
+        <x:v>https://doi.org/10.1088/2058-9565/adbf43</x:v>
       </x:c>
       <x:c r="F10" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -725,19 +725,19 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>Multiclass seismic damage detection of buildings using quantum convolutional neural network</x:v>
+        <x:v>Computation-efficient quantum convolutional neural networks for autonomous driving applications</x:v>
       </x:c>
       <x:c r="B11" s="2" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>Computer‐Aided Civil and Infrastructure Engineering</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
-        <x:v>Bhatta, Sanjeev, and Ji Dang.</x:v>
+        <x:v>Emily Jimin Roh; Chaemoon Im; Wonjun Jeong; Soohyun Park</x:v>
       </x:c>
       <x:c r="E11" s="2" t="str">
-        <x:v>https://onlinelibrary.wiley.com/doi/full/10.1111/mice.13084</x:v>
+        <x:v>https://doi.org/10.1007/s11227-025-07507-0</x:v>
       </x:c>
       <x:c r="F11" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -745,364 +745,364 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="str">
+        <x:v>A multi-topology quantum convolutional neural network with qubit-measurement attention for image classification</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>QingShan Wu; WenJie Liu; XinRan Li; Zhaofeng Su; Jian Lei</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>https://doi.org/10.1016/j.engappai.2025.111705</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="str">
+        <x:v>A Distributed Hybrid Quantum Convolutional Neural Network for Medical Image Classification</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>Yangyang Li; Zhengya Qi; Yuelin Li; Haorui Yang; Ronghua Shang; Licheng Jiao</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2501.06225</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="str">
+        <x:v>Hybrid Vision Transformer and Quantum Convolutional Neural Network for Image Classification</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="str">
+        <x:v>Mingzhu Wang; Yun Shang</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2510.12291</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="str">
+        <x:v>Efficient Gate-Encoded Quantum Convolutional Neural Network with Channel Attention for Image Classification</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>Yongzhe Lin; Guanting Yu; Tianze Zhu; Xiaofeng Jiang</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="str">
+        <x:v>https://doi.org/10.1109/ICTAI66417.2025.00079</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="str">
+        <x:v>Quantum convolutional neural network based on variational quantum circuits.</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>Optics Communications</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="str">
+        <x:v>Gong, Li-Hua, et al.</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0030401823007411</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="str">
+        <x:v>Quantum Convolutional Neural Networks are (Effectively) Classically Simulable</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>Bermejo, Pablo, et al.</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str">
+        <x:v>https://arxiv.org/pdf/2408.12739</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="str">
+        <x:v>Multiclass seismic damage detection of buildings using quantum convolutional neural network</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>Computer‐Aided Civil and Infrastructure Engineering</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Bhatta, Sanjeev, and Ji Dang.</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>https://onlinelibrary.wiley.com/doi/full/10.1111/mice.13084</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="str">
         <x:v>Optimizing Quantum Convolutional Neural Network Architectures for Arbitrary Data Dimension
 </x:v>
       </x:c>
-      <x:c r="B12" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C12" s="2" t="str">
+      <x:c r="B19" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D12" s="2" t="str">
+      <x:c r="D19" s="2" t="str">
         <x:v>Lee, Changwon, et al.</x:v>
       </x:c>
-      <x:c r="E12" s="2" t="str">
+      <x:c r="E19" s="2" t="str">
         <x:v>https://arxiv.org/pdf/2403.19099</x:v>
       </x:c>
-      <x:c r="F12" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="2" t="str">
+      <x:c r="F19" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="str">
         <x:v>Permutation-equivariant quantum convolutional neural networks
 </x:v>
       </x:c>
-      <x:c r="B13" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C13" s="2" t="str">
+      <x:c r="B20" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D13" s="2" t="str">
+      <x:c r="D20" s="2" t="str">
         <x:v>Das, Sreetama, and Filippo Caruso.</x:v>
       </x:c>
-      <x:c r="E13" s="2" t="str">
+      <x:c r="E20" s="2" t="str">
         <x:v>https://arxiv.org/abs/2404.18198</x:v>
       </x:c>
-      <x:c r="F13" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="2" t="str">
+      <x:c r="F20" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="str">
         <x:v>A New Quantum Circuits of Quantum Convolutional Neural Network for X-Ray Images Classification</x:v>
       </x:c>
-      <x:c r="B14" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C14" s="2" t="str">
+      <x:c r="B21" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
         <x:v>IEEE Access</x:v>
       </x:c>
-      <x:c r="D14" s="2" t="str">
+      <x:c r="D21" s="2" t="str">
         <x:v>Yousif, Mohammed, Belal Al-Khateeb, and Begonya Garcia-Zapirain.</x:v>
       </x:c>
-      <x:c r="E14" s="2" t="str">
+      <x:c r="E21" s="2" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10517587</x:v>
       </x:c>
-      <x:c r="F14" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2" t="str">
+      <x:c r="F21" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="str">
         <x:v>Error-tolerant quantum convolutional neural networks for symmetry-protected topological phases</x:v>
       </x:c>
-      <x:c r="B15" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C15" s="2" t="str">
+      <x:c r="B22" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
         <x:v>Physical Review Research</x:v>
       </x:c>
-      <x:c r="D15" s="2" t="str">
+      <x:c r="D22" s="2" t="str">
         <x:v>Zapletal, Petr, Nathan A. McMahon, and Michael J. Hartmann.</x:v>
       </x:c>
-      <x:c r="E15" s="2" t="str">
+      <x:c r="E22" s="2" t="str">
         <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.033111</x:v>
       </x:c>
-      <x:c r="F15" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2" t="str">
+      <x:c r="F22" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="str">
         <x:v>Splitting and parallelizing of quantum convolutional neural networks for learning translationally symmetric data</x:v>
       </x:c>
-      <x:c r="B16" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C16" s="2" t="str">
+      <x:c r="B23" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
         <x:v>Physical Review Research</x:v>
       </x:c>
-      <x:c r="D16" s="2" t="str">
+      <x:c r="D23" s="2" t="str">
         <x:v>Chinzei, Koki, et al.</x:v>
       </x:c>
-      <x:c r="E16" s="2" t="str">
+      <x:c r="E23" s="2" t="str">
         <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.023042</x:v>
       </x:c>
-      <x:c r="F16" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="2" t="str">
+      <x:c r="F23" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="str">
         <x:v>Channel attention for quantum convolutional neural networks
 </x:v>
       </x:c>
-      <x:c r="B17" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C17" s="2" t="str">
+      <x:c r="B24" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
         <x:v>Physical Review A</x:v>
       </x:c>
-      <x:c r="D17" s="2" t="str">
+      <x:c r="D24" s="2" t="str">
         <x:v>Budiutama, Gekko, et al.</x:v>
       </x:c>
-      <x:c r="E17" s="2" t="str">
+      <x:c r="E24" s="2" t="str">
         <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.110.012447</x:v>
       </x:c>
-      <x:c r="F17" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2" t="str">
+      <x:c r="F24" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="str">
         <x:v>Heart disease prediction: Improved quantum convolutional neural network and enhanced features</x:v>
       </x:c>
-      <x:c r="B18" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C18" s="2" t="str">
+      <x:c r="B25" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
         <x:v>Expert Systems with Applications </x:v>
       </x:c>
-      <x:c r="D18" s="2" t="str">
+      <x:c r="D25" s="2" t="str">
         <x:v>Pitchal, Padmakumari, Shanthi Ponnusamy, and Vidivelli Soundararajan.</x:v>
       </x:c>
-      <x:c r="E18" s="2" t="str">
+      <x:c r="E25" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417424003993</x:v>
       </x:c>
-      <x:c r="F18" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="2" t="str">
+      <x:c r="F25" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="str">
         <x:v>A resource-efficient quantum convolutional neural network</x:v>
       </x:c>
-      <x:c r="B19" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C19" s="2" t="str">
+      <x:c r="B26" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
         <x:v>Frontiers in Physics </x:v>
       </x:c>
-      <x:c r="D19" s="2" t="str">
+      <x:c r="D26" s="2" t="str">
         <x:v>Song, Yanqi, et al.</x:v>
       </x:c>
-      <x:c r="E19" s="2" t="str">
+      <x:c r="E26" s="2" t="str">
         <x:v>https://www.frontiersin.org/journals/physics/articles/10.3389/fphy.2024.1362690/full</x:v>
       </x:c>
-      <x:c r="F19" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2" t="str">
+      <x:c r="F26" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="str">
         <x:v>Shallow hybrid quantum-classical convolutional neural network model for image classification
 </x:v>
       </x:c>
-      <x:c r="B20" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C20" s="2" t="str">
+      <x:c r="B27" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
         <x:v>Quantum Information Processing </x:v>
       </x:c>
-      <x:c r="D20" s="2" t="str">
+      <x:c r="D27" s="2" t="str">
         <x:v>Wang, Aijuan, et al.</x:v>
       </x:c>
-      <x:c r="E20" s="2" t="str">
+      <x:c r="E27" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s11128-023-04217-5</x:v>
       </x:c>
-      <x:c r="F20" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2" t="str">
+      <x:c r="F27" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="str">
         <x:v>Quantum convolutional neural networks with interaction layers for classification of classical data</x:v>
       </x:c>
-      <x:c r="B21" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C21" s="2" t="str">
+      <x:c r="B28" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
         <x:v>Quantum Machine Intelligence </x:v>
       </x:c>
-      <x:c r="D21" s="2" t="str">
+      <x:c r="D28" s="2" t="str">
         <x:v>Mahmud, Jishnu, et al.</x:v>
       </x:c>
-      <x:c r="E21" s="2" t="str">
+      <x:c r="E28" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s42484-024-00145-4</x:v>
       </x:c>
-      <x:c r="F21" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="2" t="str">
+      <x:c r="F28" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="str">
         <x:v>Digital-analog quantum convolutional neural networks for image classification
 </x:v>
       </x:c>
-      <x:c r="B22" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C22" s="2" t="str">
+      <x:c r="B29" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D22" s="2" t="str">
+      <x:c r="D29" s="2" t="str">
         <x:v>Simen, Anton, et al.</x:v>
       </x:c>
-      <x:c r="E22" s="2" t="str">
+      <x:c r="E29" s="2" t="str">
         <x:v>https://arxiv.org/abs/2405.00548</x:v>
-      </x:c>
-      <x:c r="F22" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="2" t="str">
-        <x:v>Identification of quantum entanglement with Siamese convolutional neural networks and semisupervised learning</x:v>
-      </x:c>
-      <x:c r="B23" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C23" s="2" t="str">
-        <x:v>Physical Review Applied </x:v>
-      </x:c>
-      <x:c r="D23" s="2" t="str">
-        <x:v>Pawłowski, Jarosław, and Mateusz Krawczyk.</x:v>
-      </x:c>
-      <x:c r="E23" s="2" t="str">
-        <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.22.014068</x:v>
-      </x:c>
-      <x:c r="F23" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="2" t="str">
-        <x:v>A quantum convolutional network and ResNet (50)-based classification architecture for the MNIST medical dataset</x:v>
-      </x:c>
-      <x:c r="B24" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C24" s="2" t="str">
-        <x:v>Biomedical Signal Processing and Control</x:v>
-      </x:c>
-      <x:c r="D24" s="2" t="str">
-        <x:v>Hassan, Esraa, et al.</x:v>
-      </x:c>
-      <x:c r="E24" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S174680942300993X</x:v>
-      </x:c>
-      <x:c r="F24" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="2" t="str">
-        <x:v>Correlated optical convolutional neural network with “quantum speedup”</x:v>
-      </x:c>
-      <x:c r="B25" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C25" s="2" t="str">
-        <x:v>Light: Science &amp; Applications </x:v>
-      </x:c>
-      <x:c r="D25" s="2" t="str">
-        <x:v>Sun, Yifan, et al.</x:v>
-      </x:c>
-      <x:c r="E25" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41377-024-01376-7</x:v>
-      </x:c>
-      <x:c r="F25" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="2" t="str">
-        <x:v>Quantum convolutional neural networks for multiclass image classification</x:v>
-      </x:c>
-      <x:c r="B26" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C26" s="2" t="str">
-        <x:v>Quantum Information Processing </x:v>
-      </x:c>
-      <x:c r="D26" s="2" t="str">
-        <x:v>Shi, Shangshang, et al.</x:v>
-      </x:c>
-      <x:c r="E26" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11128-024-04360-7</x:v>
-      </x:c>
-      <x:c r="F26" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="2" t="str">
-        <x:v>A Deep Quantum Convolutional Neural Network Based Facial Expression Recognition For Mental Health Analysis</x:v>
-      </x:c>
-      <x:c r="B27" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C27" s="2" t="str">
-        <x:v>IEEE Transactions on Neural Systems and Rehabilitation Engineering</x:v>
-      </x:c>
-      <x:c r="D27" s="2" t="str">
-        <x:v>Hossain, Sanoar, et al.</x:v>
-      </x:c>
-      <x:c r="E27" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10491351</x:v>
-      </x:c>
-      <x:c r="F27" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="2" t="str">
-        <x:v>Harnessing quantum power using hybrid quantum deep neural network for advanced image taxonomy</x:v>
-      </x:c>
-      <x:c r="B28" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C28" s="2" t="str">
-        <x:v>Optical and Quantum Electronics</x:v>
-      </x:c>
-      <x:c r="D28" s="2" t="str">
-        <x:v>Kiran, Ajmeera, et al.</x:v>
-      </x:c>
-      <x:c r="E28" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11082-023-06202-9</x:v>
-      </x:c>
-      <x:c r="F28" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="2" t="str">
-        <x:v>HQDCNet: Hybrid Quantum Dilated Convolution Neural Network for detecting covid-19 in the context of Big Data Analytics</x:v>
-      </x:c>
-      <x:c r="B29" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C29" s="2" t="str">
-        <x:v>Multimedia Tools and Applications</x:v>
-      </x:c>
-      <x:c r="D29" s="2" t="str">
-        <x:v>Tenali, Nagamani, and Gatram Rama Mohan Babu.</x:v>
-      </x:c>
-      <x:c r="E29" s="2" t="str">
-        <x:v>https://www.ncbi.nlm.nih.gov/pmc/articles/PMC10176300/</x:v>
       </x:c>
       <x:c r="F29" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1110,201 +1110,201 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="str">
+        <x:v>Identification of quantum entanglement with Siamese convolutional neural networks and semisupervised learning</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>Physical Review Applied </x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>Pawłowski, Jarosław, and Mateusz Krawczyk.</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.22.014068</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="str">
+        <x:v>A quantum convolutional network and ResNet (50)-based classification architecture for the MNIST medical dataset</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>Biomedical Signal Processing and Control</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>Hassan, Esraa, et al.</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S174680942300993X</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="str">
+        <x:v>Correlated optical convolutional neural network with “quantum speedup”</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>Light: Science &amp; Applications </x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>Sun, Yifan, et al.</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str">
+        <x:v>https://www.nature.com/articles/s41377-024-01376-7</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="str">
+        <x:v>Quantum convolutional neural networks for multiclass image classification</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>Quantum Information Processing </x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="str">
+        <x:v>Shi, Shangshang, et al.</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11128-024-04360-7</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="str">
+        <x:v>A Deep Quantum Convolutional Neural Network Based Facial Expression Recognition For Mental Health Analysis</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>IEEE Transactions on Neural Systems and Rehabilitation Engineering</x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="str">
+        <x:v>Hossain, Sanoar, et al.</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10491351</x:v>
+      </x:c>
+      <x:c r="F34" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="str">
+        <x:v>Harnessing quantum power using hybrid quantum deep neural network for advanced image taxonomy</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>Optical and Quantum Electronics</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="str">
+        <x:v>Kiran, Ajmeera, et al.</x:v>
+      </x:c>
+      <x:c r="E35" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11082-023-06202-9</x:v>
+      </x:c>
+      <x:c r="F35" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="str">
+        <x:v>HQDCNet: Hybrid Quantum Dilated Convolution Neural Network for detecting covid-19 in the context of Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>Multimedia Tools and Applications</x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="str">
+        <x:v>Tenali, Nagamani, and Gatram Rama Mohan Babu.</x:v>
+      </x:c>
+      <x:c r="E36" s="2" t="str">
+        <x:v>https://www.ncbi.nlm.nih.gov/pmc/articles/PMC10176300/</x:v>
+      </x:c>
+      <x:c r="F36" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="str">
         <x:v>ResQuNNs:Towards Enabling Deep Learning in Quantum Convolution Neural Networks
 </x:v>
       </x:c>
-      <x:c r="B30" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C30" s="2" t="str">
+      <x:c r="B37" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D30" s="2" t="str">
+      <x:c r="D37" s="2" t="str">
         <x:v>Kashif, Muhammad, and Muhammad Shafique.</x:v>
       </x:c>
-      <x:c r="E30" s="2" t="str">
+      <x:c r="E37" s="2" t="str">
         <x:v>https://arxiv.org/pdf/2402.09146</x:v>
       </x:c>
-      <x:c r="F30" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="2" t="str">
+      <x:c r="F37" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="str">
         <x:v>XpookyNet: advancement in quantum system analysis through convolutional neural networks for detection of entanglement</x:v>
       </x:c>
-      <x:c r="B31" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C31" s="2" t="str">
+      <x:c r="B38" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
         <x:v>Quantum Machine Intelligence </x:v>
       </x:c>
-      <x:c r="D31" s="2" t="str">
+      <x:c r="D38" s="2" t="str">
         <x:v>Kookani, Ali, et al.</x:v>
       </x:c>
-      <x:c r="E31" s="2" t="str">
+      <x:c r="E38" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s42484-024-00183-y</x:v>
       </x:c>
-      <x:c r="F31" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="2" t="str">
+      <x:c r="F38" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2" t="str">
         <x:v>Brain Tumor Diagnosis Using Quantum Convolutional Neural Networks
 </x:v>
       </x:c>
-      <x:c r="B32" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C32" s="2" t="str">
+      <x:c r="B39" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D32" s="2" t="str">
+      <x:c r="D39" s="2" t="str">
         <x:v>Khan, Muhammad Al-Zafar, et al.</x:v>
       </x:c>
-      <x:c r="E32" s="2" t="str">
+      <x:c r="E39" s="2" t="str">
         <x:v>https://arxiv.org/pdf/2401.15804</x:v>
-      </x:c>
-      <x:c r="F32" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="2" t="str">
-        <x:v>A degressive quantum convolutional neural network for quantum state classification and code recognition</x:v>
-      </x:c>
-      <x:c r="B33" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C33" s="2" t="str">
-        <x:v>Iscience</x:v>
-      </x:c>
-      <x:c r="D33" s="2" t="str">
-        <x:v>Wu, Qingshan, et al.</x:v>
-      </x:c>
-      <x:c r="E33" s="2" t="str">
-        <x:v>https://www.cell.com/iscience/fulltext/S2589-0042(24)00615-1</x:v>
-      </x:c>
-      <x:c r="F33" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="2" t="str">
-        <x:v>Recognition and Classification of Concrete Surface Cracks with an Inception Quantum Convolutional Neural Network Algorithm</x:v>
-      </x:c>
-      <x:c r="B34" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C34" s="2" t="str">
-        <x:v>Applied Geophysics </x:v>
-      </x:c>
-      <x:c r="D34" s="2" t="str">
-        <x:v>Bu, Yun-zhe, et al.</x:v>
-      </x:c>
-      <x:c r="E34" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11770-024-1101-z</x:v>
-      </x:c>
-      <x:c r="F34" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="2" t="str">
-        <x:v>Quantum convolution neural network for multi-nutrient detection and stress identification in plant leaves</x:v>
-      </x:c>
-      <x:c r="B35" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C35" s="2" t="str">
-        <x:v>Multimedia Tools and Applications</x:v>
-      </x:c>
-      <x:c r="D35" s="2" t="str">
-        <x:v>Venkatesh, Kummari, K. Jairam Naik, and Achyut Shankar.</x:v>
-      </x:c>
-      <x:c r="E35" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11042-023-17992-1</x:v>
-      </x:c>
-      <x:c r="F35" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="2" t="str">
-        <x:v>Quantum-inspired activation functions in the convolutional neural network.</x:v>
-      </x:c>
-      <x:c r="B36" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C36" s="2" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D36" s="2" t="str">
-        <x:v>Li, Shaozhi, et al.</x:v>
-      </x:c>
-      <x:c r="E36" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2404.05901</x:v>
-      </x:c>
-      <x:c r="F36" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="2" t="str">
-        <x:v>Fourier Series Guided Design of Quantum Convolutional Neural Networks for Enhanced Time Series Forecasting</x:v>
-      </x:c>
-      <x:c r="B37" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C37" s="2" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D37" s="2" t="str">
-        <x:v>Osorio, Sandra Leticia Juárez, et al.</x:v>
-      </x:c>
-      <x:c r="E37" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2404.15377</x:v>
-      </x:c>
-      <x:c r="F37" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="2" t="str">
-        <x:v>Analysis of learnability of a novel hybrid quantum–classical convolutional neural network in image classification</x:v>
-      </x:c>
-      <x:c r="B38" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C38" s="2" t="str">
-        <x:v>Chinese Physics</x:v>
-      </x:c>
-      <x:c r="D38" s="2" t="str">
-        <x:v>Cheng, Tao, et al.</x:v>
-      </x:c>
-      <x:c r="E38" s="2" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/1674-1056/ad1926/meta</x:v>
-      </x:c>
-      <x:c r="F38" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="2" t="str">
-        <x:v>Handwritten digit recognition using quantum convolution neural network.</x:v>
-      </x:c>
-      <x:c r="B39" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C39" s="2" t="str">
-        <x:v>Int J Artif Intell </x:v>
-      </x:c>
-      <x:c r="D39" s="2" t="str">
-        <x:v>Daniel, Ravuri, et al.</x:v>
-      </x:c>
-      <x:c r="E39" s="2" t="str">
-        <x:v>https://pdfs.semanticscholar.org/0227/c8e0d34c276a10e9a29e5604c6ce42a26290.pdf</x:v>
       </x:c>
       <x:c r="F39" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1312,19 +1312,19 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="2" t="str">
-        <x:v>Automatic Classification of Tables Using Hybrid Quantum Convolutional Neural Networks." Intelligent Quantum Information Processing. </x:v>
+        <x:v>A degressive quantum convolutional neural network for quantum state classification and code recognition</x:v>
       </x:c>
       <x:c r="B40" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C40" s="2" t="str">
-        <x:v>Intelligent Quantum Information Processing. CRC Press</x:v>
+        <x:v>Iscience</x:v>
       </x:c>
       <x:c r="D40" s="2" t="str">
-        <x:v>Franco-Gaona, Erick, Iván Cruz-Aceves, and Maria-Susana Avila-Garcia.</x:v>
+        <x:v>Wu, Qingshan, et al.</x:v>
       </x:c>
       <x:c r="E40" s="2" t="str">
-        <x:v>https://www.taylorfrancis.com/chapters/edit/10.1201/9781003373117-3/automatic-classification-tables-using-hybrid-quantum-convolutional-neural-networks-erick-franco-gaona-iv%C3%A1n-cruz-aceves-maria-susana-avila-garcia</x:v>
+        <x:v>https://www.cell.com/iscience/fulltext/S2589-0042(24)00615-1</x:v>
       </x:c>
       <x:c r="F40" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1332,179 +1332,181 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="2" t="str">
+        <x:v>Recognition and Classification of Concrete Surface Cracks with an Inception Quantum Convolutional Neural Network Algorithm</x:v>
+      </x:c>
+      <x:c r="B41" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C41" s="2" t="str">
+        <x:v>Applied Geophysics </x:v>
+      </x:c>
+      <x:c r="D41" s="2" t="str">
+        <x:v>Bu, Yun-zhe, et al.</x:v>
+      </x:c>
+      <x:c r="E41" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11770-024-1101-z</x:v>
+      </x:c>
+      <x:c r="F41" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="2" t="str">
+        <x:v>Quantum convolution neural network for multi-nutrient detection and stress identification in plant leaves</x:v>
+      </x:c>
+      <x:c r="B42" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C42" s="2" t="str">
+        <x:v>Multimedia Tools and Applications</x:v>
+      </x:c>
+      <x:c r="D42" s="2" t="str">
+        <x:v>Venkatesh, Kummari, K. Jairam Naik, and Achyut Shankar.</x:v>
+      </x:c>
+      <x:c r="E42" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11042-023-17992-1</x:v>
+      </x:c>
+      <x:c r="F42" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2" t="str">
+        <x:v>Quantum-inspired activation functions in the convolutional neural network.</x:v>
+      </x:c>
+      <x:c r="B43" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C43" s="2" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D43" s="2" t="str">
+        <x:v>Li, Shaozhi, et al.</x:v>
+      </x:c>
+      <x:c r="E43" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2404.05901</x:v>
+      </x:c>
+      <x:c r="F43" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2" t="str">
+        <x:v>Fourier Series Guided Design of Quantum Convolutional Neural Networks for Enhanced Time Series Forecasting</x:v>
+      </x:c>
+      <x:c r="B44" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C44" s="2" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D44" s="2" t="str">
+        <x:v>Osorio, Sandra Leticia Juárez, et al.</x:v>
+      </x:c>
+      <x:c r="E44" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2404.15377</x:v>
+      </x:c>
+      <x:c r="F44" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2" t="str">
+        <x:v>Analysis of learnability of a novel hybrid quantum–classical convolutional neural network in image classification</x:v>
+      </x:c>
+      <x:c r="B45" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C45" s="2" t="str">
+        <x:v>Chinese Physics</x:v>
+      </x:c>
+      <x:c r="D45" s="2" t="str">
+        <x:v>Cheng, Tao, et al.</x:v>
+      </x:c>
+      <x:c r="E45" s="2" t="str">
+        <x:v>https://iopscience.iop.org/article/10.1088/1674-1056/ad1926/meta</x:v>
+      </x:c>
+      <x:c r="F45" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2" t="str">
+        <x:v>Handwritten digit recognition using quantum convolution neural network.</x:v>
+      </x:c>
+      <x:c r="B46" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C46" s="2" t="str">
+        <x:v>Int J Artif Intell </x:v>
+      </x:c>
+      <x:c r="D46" s="2" t="str">
+        <x:v>Daniel, Ravuri, et al.</x:v>
+      </x:c>
+      <x:c r="E46" s="2" t="str">
+        <x:v>https://pdfs.semanticscholar.org/0227/c8e0d34c276a10e9a29e5604c6ce42a26290.pdf</x:v>
+      </x:c>
+      <x:c r="F46" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2" t="str">
+        <x:v>Automatic Classification of Tables Using Hybrid Quantum Convolutional Neural Networks." Intelligent Quantum Information Processing. </x:v>
+      </x:c>
+      <x:c r="B47" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
+        <x:v>Intelligent Quantum Information Processing. CRC Press</x:v>
+      </x:c>
+      <x:c r="D47" s="2" t="str">
+        <x:v>Franco-Gaona, Erick, Iván Cruz-Aceves, and Maria-Susana Avila-Garcia.</x:v>
+      </x:c>
+      <x:c r="E47" s="2" t="str">
+        <x:v>https://www.taylorfrancis.com/chapters/edit/10.1201/9781003373117-3/automatic-classification-tables-using-hybrid-quantum-convolutional-neural-networks-erick-franco-gaona-iv%C3%A1n-cruz-aceves-maria-susana-avila-garcia</x:v>
+      </x:c>
+      <x:c r="F47" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="str">
         <x:v>Fourier Series Guided Design of Quantum Convolutional Neural Networks for Enhanced Time Series Forecasting
 </x:v>
       </x:c>
-      <x:c r="B41" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C41" s="2" t="str">
+      <x:c r="B48" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C48" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D41" s="2" t="str">
+      <x:c r="D48" s="2" t="str">
         <x:v>Osorio, Sandra Leticia Juárez, et al.</x:v>
       </x:c>
-      <x:c r="E41" s="2" t="str">
+      <x:c r="E48" s="2" t="str">
         <x:v>https://arxiv.org/abs/2404.15377</x:v>
       </x:c>
-      <x:c r="F41" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="2" t="str">
+      <x:c r="F48" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="str">
         <x:v>QuCNet: Quantum-Inspired Convolutional Neural Networks for Optimized Thyroid Nodule Classification
 </x:v>
       </x:c>
-      <x:c r="B42" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C42" s="2" t="str">
+      <x:c r="B49" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C49" s="2" t="str">
         <x:v>IEEE Access</x:v>
       </x:c>
-      <x:c r="D42" s="2" t="str">
+      <x:c r="D49" s="2" t="str">
         <x:v>Swathi, Gunti, Ali Altalbe, and R. Prasanna Kumar.</x:v>
       </x:c>
-      <x:c r="E42" s="2" t="str">
+      <x:c r="E49" s="2" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10440329</x:v>
-      </x:c>
-      <x:c r="F42" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="2" t="str">
-        <x:v>Quantum Convolutional Neural Network for Image Classification</x:v>
-      </x:c>
-      <x:c r="B43" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C43" s="2" t="str">
-        <x:v>Fusion Practice and Applications</x:v>
-      </x:c>
-      <x:c r="D43" s="2" t="str">
-        <x:v>Yousif, Moahmmed, and Belal Al-Khateeb.</x:v>
-      </x:c>
-      <x:c r="E43" s="2" t="str">
-        <x:v>https://www.researchgate.net/profile/Mohammed-Al-Yousif/publication/379449800_Quantum_Convolutional_Neural_Network_for_Image_Classification/links/660aa058390c214cfd2f2276/Quantum-Convolutional-Neural-Network-for-Image-Classification.pdf</x:v>
-      </x:c>
-      <x:c r="F43" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="2" t="str">
-        <x:v>Multi-Scale Feature Fusion Quantum Depthwise Convolutional Neural Networks for Text Classification.</x:v>
-      </x:c>
-      <x:c r="B44" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C44" s="2" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D44" s="2" t="str">
-        <x:v>Chen, Yixiong, and Weichuan Fang.</x:v>
-      </x:c>
-      <x:c r="E44" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2405.13515</x:v>
-      </x:c>
-      <x:c r="F44" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="2" t="str">
-        <x:v>Understanding the effects of data encoding on quantum-classical convolutional neural networks.</x:v>
-      </x:c>
-      <x:c r="B45" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C45" s="2" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D45" s="2" t="str">
-        <x:v>Monnet, Maureen, et al.</x:v>
-      </x:c>
-      <x:c r="E45" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2405.03027</x:v>
-      </x:c>
-      <x:c r="F45" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="2" t="str">
-        <x:v>Research on the quantum photonic convolutional neural network for artificial intelligence-based healthcare system security</x:v>
-      </x:c>
-      <x:c r="B46" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C46" s="2" t="str">
-        <x:v>Optical and Quantum Electronics </x:v>
-      </x:c>
-      <x:c r="D46" s="2" t="str">
-        <x:v>Sita Kumari, K., et al.</x:v>
-      </x:c>
-      <x:c r="E46" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11082-023-05574-2</x:v>
-      </x:c>
-      <x:c r="F46" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="2" t="str">
-        <x:v>Quantum Convolutional Neural Networks for the detection of Gamma-Ray Bursts in the AGILE space mission data</x:v>
-      </x:c>
-      <x:c r="B47" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C47" s="2" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D47" s="2" t="str">
-        <x:v>Rizzo, Alessandro, et al.</x:v>
-      </x:c>
-      <x:c r="E47" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2404.14133</x:v>
-      </x:c>
-      <x:c r="F47" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="2" t="str">
-        <x:v>Leveraging Quantum computing for synthetic image generation and recognition with Generative Adversarial Networks and Convolutional Neural Networks</x:v>
-      </x:c>
-      <x:c r="B48" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C48" s="2" t="str">
-        <x:v>International Journal of Information Technology </x:v>
-      </x:c>
-      <x:c r="D48" s="2" t="str">
-        <x:v>Golchha, Roopa, and Gyanendra K. Verma.</x:v>
-      </x:c>
-      <x:c r="E48" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s41870-024-01835-9</x:v>
-      </x:c>
-      <x:c r="F48" s="2" t="str">
-        <x:v>QCNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="2" t="str">
-        <x:v>Quantum error correction via quantum convolutional neural networks</x:v>
-      </x:c>
-      <x:c r="B49" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C49" s="2"/>
-      <x:c r="D49" s="2" t="str">
-        <x:v>Falla León, José Luis. Quantum error correction via quantum convolutional neural networks. Diss. Universidad Nacional de Colombia.</x:v>
-      </x:c>
-      <x:c r="E49" s="2" t="str">
-        <x:v>https://repositorio.unal.edu.co/handle/unal/86209</x:v>
       </x:c>
       <x:c r="F49" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1512,19 +1514,19 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="2" t="str">
-        <x:v>Model-Independent Learning of Quantum Phases of Matter with Quantum Convolutional Neural Networks</x:v>
+        <x:v>Quantum Convolutional Neural Network for Image Classification</x:v>
       </x:c>
       <x:c r="B50" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C50" s="2" t="str">
-        <x:v>APS : Physical Review A covering atomic, molecular, and optical physics and quantum science</x:v>
+        <x:v>Fusion Practice and Applications</x:v>
       </x:c>
       <x:c r="D50" s="2" t="str">
-        <x:v>Yu-Jie Liu, Adam Smith, Michael Knap, Frank Pollmann</x:v>
+        <x:v>Yousif, Moahmmed, and Belal Al-Khateeb.</x:v>
       </x:c>
       <x:c r="E50" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevLett.130.220603</x:v>
+        <x:v>https://www.researchgate.net/profile/Mohammed-Al-Yousif/publication/379449800_Quantum_Convolutional_Neural_Network_for_Image_Classification/links/660aa058390c214cfd2f2276/Quantum-Convolutional-Neural-Network-for-Image-Classification.pdf</x:v>
       </x:c>
       <x:c r="F50" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1532,19 +1534,19 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="2" t="str">
-        <x:v>Quantum convolutional neural networks for multi-channel supervised learning</x:v>
+        <x:v>Multi-Scale Feature Fusion Quantum Depthwise Convolutional Neural Networks for Text Classification.</x:v>
       </x:c>
       <x:c r="B51" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C51" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D51" s="2" t="str">
-        <x:v>Anthony M. Smaldone, Gregory W. Kyro, Victor S. Batista</x:v>
+        <x:v>Chen, Yixiong, and Weichuan Fang.</x:v>
       </x:c>
       <x:c r="E51" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00130-3</x:v>
+        <x:v>https://arxiv.org/abs/2405.13515</x:v>
       </x:c>
       <x:c r="F51" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1552,19 +1554,19 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="2" t="str">
-        <x:v>Pest Localization Using YOLOv5 and Classification Based on Quantum Convolutional Network</x:v>
+        <x:v>Understanding the effects of data encoding on quantum-classical convolutional neural networks.</x:v>
       </x:c>
       <x:c r="B52" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C52" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D52" s="2" t="str">
-        <x:v>Javeria Amin ,Muhammad Almas Anjum, Rida Zahra, Muhammad Imran Sharif, Seifedine Kadry,Lukas Sevcik</x:v>
+        <x:v>Monnet, Maureen, et al.</x:v>
       </x:c>
       <x:c r="E52" s="2" t="str">
-        <x:v>https://doi.org/10.3390/agriculture13030662</x:v>
+        <x:v>https://arxiv.org/abs/2405.03027</x:v>
       </x:c>
       <x:c r="F52" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1572,19 +1574,19 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2" t="str">
-        <x:v>Hybrid Quantum-Classical Convolutional Neural Network Model for Image Classification</x:v>
+        <x:v>Research on the quantum photonic convolutional neural network for artificial intelligence-based healthcare system security</x:v>
       </x:c>
       <x:c r="B53" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C53" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>Optical and Quantum Electronics </x:v>
       </x:c>
       <x:c r="D53" s="2" t="str">
-        <x:v>Fan Fan, Yilei Shi, Tobias Guggemos, Xiao Xiang Zhu</x:v>
+        <x:v>Sita Kumari, K., et al.</x:v>
       </x:c>
       <x:c r="E53" s="2" t="str">
-        <x:v>https://doi.org/10.1109/TNNLS.2023.3312170</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11082-023-05574-2</x:v>
       </x:c>
       <x:c r="F53" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1592,19 +1594,19 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="2" t="str">
-        <x:v>Efficient quantum feature extraction for CNN-based learning</x:v>
+        <x:v>Quantum Convolutional Neural Networks for the detection of Gamma-Ray Bursts in the AGILE space mission data</x:v>
       </x:c>
       <x:c r="B54" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C54" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D54" s="2" t="str">
-        <x:v>Fan Fan, Yilei Shi, Tobias Guggemos, Xiao Xiang Zhu</x:v>
+        <x:v>Rizzo, Alessandro, et al.</x:v>
       </x:c>
       <x:c r="E54" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.jfranklin.2023.06.003</x:v>
+        <x:v>https://arxiv.org/abs/2404.14133</x:v>
       </x:c>
       <x:c r="F54" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1612,19 +1614,19 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="2" t="str">
-        <x:v>Detection of anomaly in surveillance videos using quantum convolutional neural networks</x:v>
+        <x:v>Leveraging Quantum computing for synthetic image generation and recognition with Generative Adversarial Networks and Convolutional Neural Networks</x:v>
       </x:c>
       <x:c r="B55" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C55" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>International Journal of Information Technology </x:v>
       </x:c>
       <x:c r="D55" s="2" t="str">
-        <x:v>Javaria Amin, Muhammad Almas Anjum, Kainat Ibrar, Muhammad Sharif, Seifedine Kadry , Ruben González Cresp</x:v>
+        <x:v>Golchha, Roopa, and Gyanendra K. Verma.</x:v>
       </x:c>
       <x:c r="E55" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.imavis.2023.104710</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s41870-024-01835-9</x:v>
       </x:c>
       <x:c r="F55" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1632,19 +1634,17 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="2" t="str">
-        <x:v>Quantum cryptography in Convolution neural network approach in Smart cities</x:v>
+        <x:v>Quantum error correction via quantum convolutional neural networks</x:v>
       </x:c>
       <x:c r="B56" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C56" s="2" t="str">
-        <x:v>Journal of Survey in Fisheries Sciences</x:v>
-      </x:c>
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C56" s="2"/>
       <x:c r="D56" s="2" t="str">
-        <x:v>Nomaan Jaweed Mohammed</x:v>
+        <x:v>Falla León, José Luis. Quantum error correction via quantum convolutional neural networks. Diss. Universidad Nacional de Colombia.</x:v>
       </x:c>
       <x:c r="E56" s="2" t="str">
-        <x:v>https://doi.org/10.17762/sfs.v10i2S.1105</x:v>
+        <x:v>https://repositorio.unal.edu.co/handle/unal/86209</x:v>
       </x:c>
       <x:c r="F56" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1652,19 +1652,19 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="2" t="str">
-        <x:v>Detection of brain cancer using quantum-classical CNN-based method</x:v>
+        <x:v>Model-Independent Learning of Quantum Phases of Matter with Quantum Convolutional Neural Networks</x:v>
       </x:c>
       <x:c r="B57" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C57" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>APS : Physical Review A covering atomic, molecular, and optical physics and quantum science</x:v>
       </x:c>
       <x:c r="D57" s="2" t="str">
-        <x:v>Sriya Bada, Sreeraj Rajan Warrier, Jayasri Dontabhaktuni</x:v>
+        <x:v>Yu-Jie Liu, Adam Smith, Michael Knap, Frank Pollmann</x:v>
       </x:c>
       <x:c r="E57" s="2" t="str">
-        <x:v>https://doi.org/10.1117/12.2650132</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevLett.130.220603</x:v>
       </x:c>
       <x:c r="F57" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1672,7 +1672,7 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="2" t="str">
-        <x:v>Medical image diagnosis based on adaptive Hybrid Quantum CNN</x:v>
+        <x:v>Quantum convolutional neural networks for multi-channel supervised learning</x:v>
       </x:c>
       <x:c r="B58" s="2" t="n">
         <x:v>2023</x:v>
@@ -1681,10 +1681,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D58" s="2" t="str">
-        <x:v>Naim Ajlouni, Adem Özyavaş, Mustafa Takaoğlu, Faruk Takaoğlu &amp; Firas Ajlouni </x:v>
+        <x:v>Anthony M. Smaldone, Gregory W. Kyro, Victor S. Batista</x:v>
       </x:c>
       <x:c r="E58" s="2" t="str">
-        <x:v>https://doi.org/10.1186/s12880-023-01084-5</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00130-3</x:v>
       </x:c>
       <x:c r="F58" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1692,19 +1692,19 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="2" t="str">
-        <x:v>Early-stage esophageal cancer detection using hybrid quantum CNN</x:v>
+        <x:v>Pest Localization Using YOLOv5 and Classification Based on Quantum Convolutional Network</x:v>
       </x:c>
       <x:c r="B59" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C59" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str">
-        <x:v>R. I. Minu, Martin Margala, S. Siva Shankar, Prasun Chakrabarti &amp; G. Nagarajan</x:v>
+        <x:v>Javeria Amin ,Muhammad Almas Anjum, Rida Zahra, Muhammad Imran Sharif, Seifedine Kadry,Lukas Sevcik</x:v>
       </x:c>
       <x:c r="E59" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s00500-023-08333-3</x:v>
+        <x:v>https://doi.org/10.3390/agriculture13030662</x:v>
       </x:c>
       <x:c r="F59" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1712,19 +1712,19 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="2" t="str">
-        <x:v>Remote Sensing Image Scene Classification in Hybrid Classical–Quantum Transferring CNN with Small Samples</x:v>
+        <x:v>Hybrid Quantum-Classical Convolutional Neural Network Model for Image Classification</x:v>
       </x:c>
       <x:c r="B60" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C60" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D60" s="2" t="str">
-        <x:v> Zhouwei Zhang ,Xiaofei Mi ,Jian Yang ,Xiangqin Wei ,Yan Liu,Jian Yan ,Peizhuo Liu ,Xingfa Gu  and Tao Yu </x:v>
+        <x:v>Fan Fan, Yilei Shi, Tobias Guggemos, Xiao Xiang Zhu</x:v>
       </x:c>
       <x:c r="E60" s="2" t="str">
-        <x:v>https://doi.org/10.3390/s23188010</x:v>
+        <x:v>https://doi.org/10.1109/TNNLS.2023.3312170</x:v>
       </x:c>
       <x:c r="F60" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1732,19 +1732,19 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="2" t="str">
-        <x:v>Hybrid Quantum Convolutional Neural Networks for UWB Signal Classification</x:v>
+        <x:v>Efficient quantum feature extraction for CNN-based learning</x:v>
       </x:c>
       <x:c r="B61" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C61" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D61" s="2" t="str">
-        <x:v>Seon-Geun Jeong; Quang-Vinh Do; Hae-Ji Hwang; Mikio Hasegawa; Hiroo Sekiya; Won-Joo Hwang</x:v>
+        <x:v>Fan Fan, Yilei Shi, Tobias Guggemos, Xiao Xiang Zhu</x:v>
       </x:c>
       <x:c r="E61" s="2" t="str">
-        <x:v>https://doi.org/10.1109/ACCESS.2023.3323019</x:v>
+        <x:v>https://doi.org/10.1016/j.jfranklin.2023.06.003</x:v>
       </x:c>
       <x:c r="F61" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1752,19 +1752,19 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="2" t="str">
-        <x:v>A Quantum Convolutional Neural Network Approach for Object Detection and Classification</x:v>
+        <x:v>Detection of anomaly in surveillance videos using quantum convolutional neural networks</x:v>
       </x:c>
       <x:c r="B62" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C62" s="2" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D62" s="2" t="str">
-        <x:v>Gowri Namratha Meedinti, Kandukuri Sai Srirekha, Radhakrishnan Delhibabu</x:v>
+        <x:v>Javaria Amin, Muhammad Almas Anjum, Kainat Ibrar, Muhammad Sharif, Seifedine Kadry , Ruben González Cresp</x:v>
       </x:c>
       <x:c r="E62" s="2" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2307.08204</x:v>
+        <x:v>https://doi.org/10.1016/j.imavis.2023.104710</x:v>
       </x:c>
       <x:c r="F62" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1772,19 +1772,19 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="2" t="str">
-        <x:v>Stereoscopic scalable quantum convolutional neural networks</x:v>
+        <x:v>Quantum cryptography in Convolution neural network approach in Smart cities</x:v>
       </x:c>
       <x:c r="B63" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C63" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>Journal of Survey in Fisheries Sciences</x:v>
       </x:c>
       <x:c r="D63" s="2" t="str">
-        <x:v>Hankyul Baek, Won Joon Yun, Soohyun Park, Joongheon Kim</x:v>
+        <x:v>Nomaan Jaweed Mohammed</x:v>
       </x:c>
       <x:c r="E63" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.neunet.2023.06.027</x:v>
+        <x:v>https://doi.org/10.17762/sfs.v10i2S.1105</x:v>
       </x:c>
       <x:c r="F63" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1792,7 +1792,7 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="2" t="str">
-        <x:v>Image classification and adversarial robustness analysis based on hybrid quantum–classical convolutional neural network</x:v>
+        <x:v>Detection of brain cancer using quantum-classical CNN-based method</x:v>
       </x:c>
       <x:c r="B64" s="2" t="n">
         <x:v>2023</x:v>
@@ -1801,10 +1801,10 @@
         <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D64" s="2" t="str">
-        <x:v>Shui-Yuan Huang, Wan-Jia An , De-Shun Zhang , Nan-Run Zhou</x:v>
+        <x:v>Sriya Bada, Sreeraj Rajan Warrier, Jayasri Dontabhaktuni</x:v>
       </x:c>
       <x:c r="E64" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.optcom.2023.129287</x:v>
+        <x:v>https://doi.org/10.1117/12.2650132</x:v>
       </x:c>
       <x:c r="F64" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1812,7 +1812,7 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="2" t="str">
-        <x:v>QSurfNet: a hybrid quantum convolutional neural network for surface defect recognition</x:v>
+        <x:v>Medical image diagnosis based on adaptive Hybrid Quantum CNN</x:v>
       </x:c>
       <x:c r="B65" s="2" t="n">
         <x:v>2023</x:v>
@@ -1821,10 +1821,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D65" s="2" t="str">
-        <x:v>Shraddha Mishra &amp; Chi-Yi Tsai</x:v>
+        <x:v>Naim Ajlouni, Adem Özyavaş, Mustafa Takaoğlu, Faruk Takaoğlu &amp; Firas Ajlouni </x:v>
       </x:c>
       <x:c r="E65" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s11128-023-03930-5</x:v>
+        <x:v>https://doi.org/10.1186/s12880-023-01084-5</x:v>
       </x:c>
       <x:c r="F65" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1832,19 +1832,19 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="2" t="str">
-        <x:v>Computational Framework of Inverted Fuzzy C-Means and Quantum Convolutional Neural Network Towards Accurate Detection of Ovarian Tumors</x:v>
+        <x:v>Early-stage esophageal cancer detection using hybrid quantum CNN</x:v>
       </x:c>
       <x:c r="B66" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C66" s="2" t="str">
-        <x:v> International Journal of E-Health and Medical Communications (IJEHMC)</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D66" s="2" t="str">
-        <x:v>Ashwini Kodipalli, Steven L. Fernandes, Santosh K. Dasar, Taha Ismail</x:v>
+        <x:v>R. I. Minu, Martin Margala, S. Siva Shankar, Prasun Chakrabarti &amp; G. Nagarajan</x:v>
       </x:c>
       <x:c r="E66" s="2" t="str">
-        <x:v>https://doi.org/10.4018/IJEHMC.321149</x:v>
+        <x:v>https://doi.org/10.1007/s00500-023-08333-3</x:v>
       </x:c>
       <x:c r="F66" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1852,19 +1852,19 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="2" t="str">
-        <x:v>QuCNN: A Quantum Convolutional Neural Network with Entanglement Based Backpropagation</x:v>
+        <x:v>Remote Sensing Image Scene Classification in Hybrid Classical–Quantum Transferring CNN with Small Samples</x:v>
       </x:c>
       <x:c r="B67" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C67" s="2" t="str">
-        <x:v>2022 IEEE/ACM</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D67" s="2" t="str">
-        <x:v>Samuel Stein; Ying Mao; James Ang; Ang Li</x:v>
+        <x:v> Zhouwei Zhang ,Xiaofei Mi ,Jian Yang ,Xiangqin Wei ,Yan Liu,Jian Yan ,Peizhuo Liu ,Xingfa Gu  and Tao Yu </x:v>
       </x:c>
       <x:c r="E67" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9996667</x:v>
+        <x:v>https://doi.org/10.3390/s23188010</x:v>
       </x:c>
       <x:c r="F67" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1872,19 +1872,19 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="2" t="str">
-        <x:v>Realizing quantum convolutional neural networks on a superconducting quantum processor to recognize quantum phases</x:v>
+        <x:v>Hybrid Quantum Convolutional Neural Networks for UWB Signal Classification</x:v>
       </x:c>
       <x:c r="B68" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C68" s="2" t="str">
-        <x:v>Nature Communications</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D68" s="2" t="str">
-        <x:v>    Johannes Herrmann, Sergi Masot Llima, Ants Remm, Petr Zapletal, Nathan A. McMahon, Colin Scarato, François Swiadek, Christian Kraglund Andersen, Christoph Hellings, Sebastian Krinner, Nathan Lacroix, Stefania Lazar, Michael Kerschbaum, Dante Colao Zanuz, Graham J. Norris, Michael J. Hartmann, Andreas Wallraff &amp; Christopher Eichler</x:v>
+        <x:v>Seon-Geun Jeong; Quang-Vinh Do; Hae-Ji Hwang; Mikio Hasegawa; Hiroo Sekiya; Won-Joo Hwang</x:v>
       </x:c>
       <x:c r="E68" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41467-022-31679-5</x:v>
+        <x:v>https://doi.org/10.1109/ACCESS.2023.3323019</x:v>
       </x:c>
       <x:c r="F68" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1892,19 +1892,19 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="2" t="str">
-        <x:v>A quantum convolutional neural network on NISQ devices</x:v>
+        <x:v>A Quantum Convolutional Neural Network Approach for Object Detection and Classification</x:v>
       </x:c>
       <x:c r="B69" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C69" s="2" t="str">
-        <x:v>AAPPS Bulletin</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D69" s="2" t="str">
-        <x:v>ShiJie Wei, YanHu Chen, ZengRong Zhou &amp; GuiLu Long</x:v>
+        <x:v>Gowri Namratha Meedinti, Kandukuri Sai Srirekha, Radhakrishnan Delhibabu</x:v>
       </x:c>
       <x:c r="E69" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s43673-021-00030-3</x:v>
+        <x:v>https://doi.org/10.48550/arXiv.2307.08204</x:v>
       </x:c>
       <x:c r="F69" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1912,19 +1912,19 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="2" t="str">
-        <x:v>Quantum convolutional neural network for classical data classification</x:v>
+        <x:v>Stereoscopic scalable quantum convolutional neural networks</x:v>
       </x:c>
       <x:c r="B70" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C70" s="2" t="str">
-        <x:v>SpringerLink</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D70" s="2" t="str">
-        <x:v>Tak Hur, Leeseok Kim &amp; Daniel K. Park</x:v>
+        <x:v>Hankyul Baek, Won Joon Yun, Soohyun Park, Joongheon Kim</x:v>
       </x:c>
       <x:c r="E70" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-021-00061-x</x:v>
+        <x:v>https://doi.org/10.1016/j.neunet.2023.06.027</x:v>
       </x:c>
       <x:c r="F70" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1932,19 +1932,19 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="2" t="str">
-        <x:v>Hybrid quantum-classical convolutional neural network model for COVID-19 prediction using chest X-ray images </x:v>
+        <x:v>Image classification and adversarial robustness analysis based on hybrid quantum–classical convolutional neural network</x:v>
       </x:c>
       <x:c r="B71" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C71" s="2" t="str">
-        <x:v>Computational Design and Engineering, 2022,</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D71" s="2" t="str">
-        <x:v>Essam H. Houssein ,  Zainab Abohashima , Mohamed Elhoseny and Waleed M. Mohamed</x:v>
+        <x:v>Shui-Yuan Huang, Wan-Jia An , De-Shun Zhang , Nan-Run Zhou</x:v>
       </x:c>
       <x:c r="E71" s="2" t="str">
-        <x:v>https://academic.oup.com/jcde/article/9/2/343/6537164</x:v>
+        <x:v>https://doi.org/10.1016/j.optcom.2023.129287</x:v>
       </x:c>
       <x:c r="F71" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1952,19 +1952,19 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="2" t="str">
-        <x:v>Scalable Quantum Convolutional Neural Networks</x:v>
+        <x:v>QSurfNet: a hybrid quantum convolutional neural network for surface defect recognition</x:v>
       </x:c>
       <x:c r="B72" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C72" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D72" s="2" t="str">
-        <x:v>Hankyul Baek, Won Joon Yun, Joongheon Kim</x:v>
+        <x:v>Shraddha Mishra &amp; Chi-Yi Tsai</x:v>
       </x:c>
       <x:c r="E72" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2209.12372</x:v>
+        <x:v>https://doi.org/10.1007/s11128-023-03930-5</x:v>
       </x:c>
       <x:c r="F72" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1972,19 +1972,19 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="2" t="str">
-        <x:v>Using a Deep Quantum Neural Network to Enhance the Fidelity of Quantum Convolutional Codes</x:v>
+        <x:v>Computational Framework of Inverted Fuzzy C-Means and Quantum Convolutional Neural Network Towards Accurate Detection of Ovarian Tumors</x:v>
       </x:c>
       <x:c r="B73" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C73" s="2" t="str">
-        <x:v>Mdpi ( Quantum Information and Quantum Computing)</x:v>
+        <x:v> International Journal of E-Health and Medical Communications (IJEHMC)</x:v>
       </x:c>
       <x:c r="D73" s="2" t="str">
-        <x:v>Hanwei Xiao, Xiaoguang Chen and Jin Xu</x:v>
+        <x:v>Ashwini Kodipalli, Steven L. Fernandes, Santosh K. Dasar, Taha Ismail</x:v>
       </x:c>
       <x:c r="E73" s="2" t="str">
-        <x:v>https://www.mdpi.com/2076-3417/12/11/5662</x:v>
+        <x:v>https://doi.org/10.4018/IJEHMC.321149</x:v>
       </x:c>
       <x:c r="F73" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -1992,19 +1992,19 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="2" t="str">
-        <x:v>Multiclass classification using quantum convolutional neural networks with hybrid quantum-classical learning</x:v>
+        <x:v>QuCNN: A Quantum Convolutional Neural Network with Entanglement Based Backpropagation</x:v>
       </x:c>
       <x:c r="B74" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C74" s="2" t="str">
-        <x:v>Sec. Quantum Engineering and Technology</x:v>
+        <x:v>2022 IEEE/ACM</x:v>
       </x:c>
       <x:c r="D74" s="2" t="str">
-        <x:v>Denis Bokhan , Alena S. Mastiukova, Aleksey S. Boev , Dmitrii N. Trubnikov and Aleksey K. Fedorov</x:v>
+        <x:v>Samuel Stein; Ying Mao; James Ang; Ang Li</x:v>
       </x:c>
       <x:c r="E74" s="2" t="str">
-        <x:v>https://www.frontiersin.org/journals/physics/articles/10.3389/fphy.2022.1069985/full</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9996667</x:v>
       </x:c>
       <x:c r="F74" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2012,19 +2012,19 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="2" t="str">
-        <x:v>An Image Classification Algorithm Based on Hybrid Quantum Classical Convolutional Neural Network</x:v>
+        <x:v>Realizing quantum convolutional neural networks on a superconducting quantum processor to recognize quantum phases</x:v>
       </x:c>
       <x:c r="B75" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C75" s="2" t="str">
-        <x:v>Quantum engineering</x:v>
+        <x:v>Nature Communications</x:v>
       </x:c>
       <x:c r="D75" s="2" t="str">
-        <x:v>Wei Li, Peng-Cheng Chu, Guang-Zhe Liu, Yan-Bing Tian, Tian-Hui Qiu, Shu-Mei Wang</x:v>
+        <x:v>    Johannes Herrmann, Sergi Masot Llima, Ants Remm, Petr Zapletal, Nathan A. McMahon, Colin Scarato, François Swiadek, Christian Kraglund Andersen, Christoph Hellings, Sebastian Krinner, Nathan Lacroix, Stefania Lazar, Michael Kerschbaum, Dante Colao Zanuz, Graham J. Norris, Michael J. Hartmann, Andreas Wallraff &amp; Christopher Eichler</x:v>
       </x:c>
       <x:c r="E75" s="2" t="str">
-        <x:v>https://onlinelibrary.wiley.com/doi/full/10.1155/2022/5701479</x:v>
+        <x:v>https://www.nature.com/articles/s41467-022-31679-5</x:v>
       </x:c>
       <x:c r="F75" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2032,19 +2032,19 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="2" t="str">
-        <x:v>Quantum ReLU activation for Convolutional Neural Networks to improve diagnosis of Parkinson’s disease and COVID-19</x:v>
+        <x:v>A quantum convolutional neural network on NISQ devices</x:v>
       </x:c>
       <x:c r="B76" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C76" s="2" t="str">
-        <x:v>Expert Systems with Applications</x:v>
+        <x:v>AAPPS Bulletin</x:v>
       </x:c>
       <x:c r="D76" s="2" t="str">
-        <x:v>Luca Parisi a b c 1, Daniel Neagu a 2, Renfei Ma b d 3, Felician Campean</x:v>
+        <x:v>ShiJie Wei, YanHu Chen, ZengRong Zhou &amp; GuiLu Long</x:v>
       </x:c>
       <x:c r="E76" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417421012483</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s43673-021-00030-3</x:v>
       </x:c>
       <x:c r="F76" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2052,19 +2052,19 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="2" t="str">
-        <x:v>Towards Explainable Quantum Machine Learning for Mobile Malware Detection and Classification</x:v>
+        <x:v>Quantum convolutional neural network for classical data classification</x:v>
       </x:c>
       <x:c r="B77" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C77" s="2" t="str">
-        <x:v>Innovation in Information Security</x:v>
+        <x:v>SpringerLink</x:v>
       </x:c>
       <x:c r="D77" s="2" t="str">
-        <x:v>Francesco Mercaldo, Giovanni Ciaramella, Giacomo Iadarola, Marco Storto, Fabio Martinelli and Antonella Santone</x:v>
+        <x:v>Tak Hur, Leeseok Kim &amp; Daniel K. Park</x:v>
       </x:c>
       <x:c r="E77" s="2" t="str">
-        <x:v>https://www.mdpi.com/2076-3417/12/23/12025</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s42484-021-00061-x</x:v>
       </x:c>
       <x:c r="F77" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2072,19 +2072,19 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="2" t="str">
-        <x:v>Quantum-classical convolutional neural networks in radiological image classification</x:v>
+        <x:v>Hybrid quantum-classical convolutional neural network model for COVID-19 prediction using chest X-ray images </x:v>
       </x:c>
       <x:c r="B78" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C78" s="2" t="str">
-        <x:v>2022 IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
+        <x:v>Computational Design and Engineering, 2022,</x:v>
       </x:c>
       <x:c r="D78" s="2" t="str">
-        <x:v>Andrea Matic; Maureen Monnet; Jeanette Miriam Lorenz; Balthasar Schachtner; Thomas Messerer</x:v>
+        <x:v>Essam H. Houssein ,  Zainab Abohashima , Mohamed Elhoseny and Waleed M. Mohamed</x:v>
       </x:c>
       <x:c r="E78" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9951255</x:v>
+        <x:v>https://academic.oup.com/jcde/article/9/2/343/6537164</x:v>
       </x:c>
       <x:c r="F78" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2092,19 +2092,19 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="2" t="str">
-        <x:v>A Novel Framework For Brain Disease Classification Using Quantum Convolutional Neural Network</x:v>
+        <x:v>Scalable Quantum Convolutional Neural Networks</x:v>
       </x:c>
       <x:c r="B79" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C79" s="2" t="str">
-        <x:v>2022 IEEE International Women in Engineering (WIE) Conference on Electrical and Computer Engineering (WIECON-ECE)</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D79" s="2" t="str">
-        <x:v>Sanskriti Chandra; Shivam Saxena; Santosh Kumar; Mithilesh Kumar Chaube; Narendra Kuber Bodhey</x:v>
+        <x:v>Hankyul Baek, Won Joon Yun, Joongheon Kim</x:v>
       </x:c>
       <x:c r="E79" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10150851</x:v>
+        <x:v>https://arxiv.org/abs/2209.12372</x:v>
       </x:c>
       <x:c r="F79" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2112,19 +2112,19 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="2" t="str">
-        <x:v>Quantum Image Classification on NISQ Devices</x:v>
+        <x:v>Using a Deep Quantum Neural Network to Enhance the Fidelity of Quantum Convolutional Codes</x:v>
       </x:c>
       <x:c r="B80" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C80" s="2" t="str">
-        <x:v>2022 14th International Conference on Computational Intelligence and Communication Networks (CICN)</x:v>
+        <x:v>Mdpi ( Quantum Information and Quantum Computing)</x:v>
       </x:c>
       <x:c r="D80" s="2" t="str">
-        <x:v>Shuroog Al-Ogbi; Abdulrahman Ashour; Muhamad Felemban</x:v>
+        <x:v>Hanwei Xiao, Xiaoguang Chen and Jin Xu</x:v>
       </x:c>
       <x:c r="E80" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10008259</x:v>
+        <x:v>https://www.mdpi.com/2076-3417/12/11/5662</x:v>
       </x:c>
       <x:c r="F80" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2132,19 +2132,19 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="2" t="str">
-        <x:v>Signal Quality Assessment of Photoplethysmogram Signals using Quantum Pattern Recognition Technique and lightweight CNN Module</x:v>
+        <x:v>Multiclass classification using quantum convolutional neural networks with hybrid quantum-classical learning</x:v>
       </x:c>
       <x:c r="B81" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C81" s="2" t="str">
-        <x:v>2022 44th Annual International Conference of the IEEE Engineering in Medicine &amp; Biology Society (EMBC)</x:v>
+        <x:v>Sec. Quantum Engineering and Technology</x:v>
       </x:c>
       <x:c r="D81" s="2" t="str">
-        <x:v>Tamaghno Chatterjee; Aayushman Ghosh; Sayan Sarkar</x:v>
+        <x:v>Denis Bokhan , Alena S. Mastiukova, Aleksey S. Boev , Dmitrii N. Trubnikov and Aleksey K. Fedorov</x:v>
       </x:c>
       <x:c r="E81" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9871494</x:v>
+        <x:v>https://www.frontiersin.org/journals/physics/articles/10.3389/fphy.2022.1069985/full</x:v>
       </x:c>
       <x:c r="F81" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2152,19 +2152,19 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="2" t="str">
-        <x:v>Quantum convolutional neural networks for high energy physics data analysis</x:v>
+        <x:v>An Image Classification Algorithm Based on Hybrid Quantum Classical Convolutional Neural Network</x:v>
       </x:c>
       <x:c r="B82" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C82" s="2" t="str">
-        <x:v>Phys. Rev. Research</x:v>
+        <x:v>Quantum engineering</x:v>
       </x:c>
       <x:c r="D82" s="2" t="str">
-        <x:v>Samuel Yen-Chi Chen, Tzu-Chieh Wei, Chao Zhang, Haiwang Yu, and Shinjae Yoo</x:v>
+        <x:v>Wei Li, Peng-Cheng Chu, Guang-Zhe Liu, Yan-Bing Tian, Tian-Hui Qiu, Shu-Mei Wang</x:v>
       </x:c>
       <x:c r="E82" s="2" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.013231</x:v>
+        <x:v>https://onlinelibrary.wiley.com/doi/full/10.1155/2022/5701479</x:v>
       </x:c>
       <x:c r="F82" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2172,19 +2172,19 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="2" t="str">
-        <x:v>Quantum-inspired complex convolutional neural networks</x:v>
+        <x:v>Quantum ReLU activation for Convolutional Neural Networks to improve diagnosis of Parkinson’s disease and COVID-19</x:v>
       </x:c>
       <x:c r="B83" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C83" s="2" t="str">
-        <x:v>Applied Intelligence</x:v>
+        <x:v>Expert Systems with Applications</x:v>
       </x:c>
       <x:c r="D83" s="2" t="str">
-        <x:v>Shangshang Shi, Zhimin Wang, Guolong Cui, Shengbin Wang, Ruimin Shang, Wendong Li, Zhiqiang Wei &amp; Yongjian Gu</x:v>
+        <x:v>Luca Parisi a b c 1, Daniel Neagu a 2, Renfei Ma b d 3, Felician Campean</x:v>
       </x:c>
       <x:c r="E83" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10489-022-03525-0</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417421012483</x:v>
       </x:c>
       <x:c r="F83" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2192,19 +2192,19 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="2" t="str">
-        <x:v>Convolutional Neural Networks (CNN) with Quantum-Behaved Particle Swarm Optimization (QPSO)-Based Medical Image Fusion</x:v>
+        <x:v>Towards Explainable Quantum Machine Learning for Mobile Malware Detection and Classification</x:v>
       </x:c>
       <x:c r="B84" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C84" s="2" t="str">
-        <x:v>Special Issue on Emerging Advances in Medical Image Computation and Computer Assisted Intervention</x:v>
+        <x:v>Innovation in Information Security</x:v>
       </x:c>
       <x:c r="D84" s="2" t="str">
-        <x:v>A. Ancy Mergin and M. S. Godwin Premi</x:v>
+        <x:v>Francesco Mercaldo, Giovanni Ciaramella, Giacomo Iadarola, Marco Storto, Fabio Martinelli and Antonella Santone</x:v>
       </x:c>
       <x:c r="E84" s="2" t="str">
-        <x:v>https://www.worldscientific.com/doi/abs/10.1142/S0219467823400053</x:v>
+        <x:v>https://www.mdpi.com/2076-3417/12/23/12025</x:v>
       </x:c>
       <x:c r="F84" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2212,19 +2212,19 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="2" t="str">
-        <x:v>Quantum Particle Swarm Optimization Based Convolutional Neural Network for Handwritten Script Recognition</x:v>
+        <x:v>Quantum-classical convolutional neural networks in radiological image classification</x:v>
       </x:c>
       <x:c r="B85" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C85" s="2" t="str">
-        <x:v>Computers Materials &amp; Continua</x:v>
+        <x:v>2022 IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
       </x:c>
       <x:c r="D85" s="2" t="str">
-        <x:v>Reya Sharma, Baijnath Kaushik, Mohammad Khalid Imam Rahmani</x:v>
+        <x:v>Andrea Matic; Maureen Monnet; Jeanette Miriam Lorenz; Balthasar Schachtner; Thomas Messerer</x:v>
       </x:c>
       <x:c r="E85" s="2" t="str">
-        <x:v>https://www.semanticscholar.org/paper/Quantum-Particle-Swarm-Optimization-Based-Neural-Sharma-Kaushik/af2936752600a75a3579b37013bb1db3220bd078?p2df</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9951255</x:v>
       </x:c>
       <x:c r="F85" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2232,19 +2232,19 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="2" t="str">
-        <x:v>Quantum Dilated Convolutional Neural Networks</x:v>
+        <x:v>A Novel Framework For Brain Disease Classification Using Quantum Convolutional Neural Network</x:v>
       </x:c>
       <x:c r="B86" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C86" s="2" t="str">
-        <x:v>IEEE Access</x:v>
+        <x:v>2022 IEEE International Women in Engineering (WIE) Conference on Electrical and Computer Engineering (WIECON-ECE)</x:v>
       </x:c>
       <x:c r="D86" s="2" t="str">
-        <x:v>Yixiong Chen</x:v>
+        <x:v>Sanskriti Chandra; Shivam Saxena; Santosh Kumar; Mithilesh Kumar Chaube; Narendra Kuber Bodhey</x:v>
       </x:c>
       <x:c r="E86" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9715107</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10150851</x:v>
       </x:c>
       <x:c r="F86" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2252,19 +2252,19 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="2" t="str">
-        <x:v>Efficient Quantum Image Classification Using Single Qubit Encoding</x:v>
+        <x:v>Quantum Image Classification on NISQ Devices</x:v>
       </x:c>
       <x:c r="B87" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C87" s="2" t="str">
-        <x:v>IEEE Transactions on Neural Networks and Learning Systems</x:v>
+        <x:v>2022 14th International Conference on Computational Intelligence and Communication Networks (CICN)</x:v>
       </x:c>
       <x:c r="D87" s="2" t="str">
-        <x:v>Philip Easom-McCaldin; Ahmed Bouridane; Ammar Belatreche; Richard Jiang; Somaya Al-Maadeed</x:v>
+        <x:v>Shuroog Al-Ogbi; Abdulrahman Ashour; Muhamad Felemban</x:v>
       </x:c>
       <x:c r="E87" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9798852</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10008259</x:v>
       </x:c>
       <x:c r="F87" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2272,19 +2272,19 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="2" t="str">
-        <x:v>Quantum-behaved particle swarm optimization of convolutional neural network for fault diagnosis</x:v>
+        <x:v>Signal Quality Assessment of Photoplethysmogram Signals using Quantum Pattern Recognition Technique and lightweight CNN Module</x:v>
       </x:c>
       <x:c r="B88" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C88" s="2" t="str">
-        <x:v>Journal of Experimental &amp; Theoretical Artificial Intelligence</x:v>
+        <x:v>2022 44th Annual International Conference of the IEEE Engineering in Medicine &amp; Biology Society (EMBC)</x:v>
       </x:c>
       <x:c r="D88" s="2" t="str">
-        <x:v>Jie Chen , QingShan Xu , Xiaofeng Xue , Yingchao Guo &amp; Runfeng Chen</x:v>
+        <x:v>Tamaghno Chatterjee; Aayushman Ghosh; Sayan Sarkar</x:v>
       </x:c>
       <x:c r="E88" s="2" t="str">
-        <x:v>https://www.tandfonline.com/doi/abs/10.1080/0952813X.2022.2120089</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9871494</x:v>
       </x:c>
       <x:c r="F88" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2292,19 +2292,19 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="2" t="str">
-        <x:v>Case study on quantum convolutional neural network scalability</x:v>
+        <x:v>Quantum convolutional neural networks for high energy physics data analysis</x:v>
       </x:c>
       <x:c r="B89" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C89" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Phys. Rev. Research</x:v>
       </x:c>
       <x:c r="D89" s="2" t="str">
-        <x:v>Marina O. Lisnichenko, Stanislav I. Protasov</x:v>
+        <x:v>Samuel Yen-Chi Chen, Tzu-Chieh Wei, Chao Zhang, Haiwang Yu, and Shinjae Yoo</x:v>
       </x:c>
       <x:c r="E89" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2207.07160</x:v>
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.013231</x:v>
       </x:c>
       <x:c r="F89" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2312,19 +2312,19 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="2" t="str">
-        <x:v>Poster: Scalable Quantum Convolutional Neural Networks for Edge Computing</x:v>
+        <x:v>Quantum-inspired complex convolutional neural networks</x:v>
       </x:c>
       <x:c r="B90" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C90" s="2" t="str">
-        <x:v>2022 IEEE/ACM 7th Symposium on Edge Computing (SEC)</x:v>
+        <x:v>Applied Intelligence</x:v>
       </x:c>
       <x:c r="D90" s="2" t="str">
-        <x:v>Jindi Wu; Qun Li</x:v>
+        <x:v>Shangshang Shi, Zhimin Wang, Guolong Cui, Shengbin Wang, Ruimin Shang, Wendong Li, Zhiqiang Wei &amp; Yongjian Gu</x:v>
       </x:c>
       <x:c r="E90" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9996801</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s10489-022-03525-0</x:v>
       </x:c>
       <x:c r="F90" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2332,19 +2332,19 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="2" t="str">
-        <x:v>A QCNN Algorithm Deployed on A Quantum Computer</x:v>
+        <x:v>Convolutional Neural Networks (CNN) with Quantum-Behaved Particle Swarm Optimization (QPSO)-Based Medical Image Fusion</x:v>
       </x:c>
       <x:c r="B91" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C91" s="2" t="str">
-        <x:v>2022 International Conference on Computing, Communication, Perception and Quantum Technology (CCPQT)</x:v>
+        <x:v>Special Issue on Emerging Advances in Medical Image Computation and Computer Assisted Intervention</x:v>
       </x:c>
       <x:c r="D91" s="2" t="str">
-        <x:v>Xinmiao Chen; Bo Jiang; Yongzheng Wu; Yongjin Ye</x:v>
+        <x:v>A. Ancy Mergin and M. S. Godwin Premi</x:v>
       </x:c>
       <x:c r="E91" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9939255</x:v>
+        <x:v>https://www.worldscientific.com/doi/abs/10.1142/S0219467823400053</x:v>
       </x:c>
       <x:c r="F91" s="2" t="str">
         <x:v>QCNN</x:v>
@@ -2352,45 +2352,185 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="2" t="str">
-        <x:v>Malaria Parasite Detection Using a Quantum-Convolutional Network</x:v>
+        <x:v>Quantum Particle Swarm Optimization Based Convolutional Neural Network for Handwritten Script Recognition</x:v>
       </x:c>
       <x:c r="B92" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C92" s="2" t="str">
+        <x:v>Computers Materials &amp; Continua</x:v>
+      </x:c>
+      <x:c r="D92" s="2" t="str">
+        <x:v>Reya Sharma, Baijnath Kaushik, Mohammad Khalid Imam Rahmani</x:v>
+      </x:c>
+      <x:c r="E92" s="2" t="str">
+        <x:v>https://www.semanticscholar.org/paper/Quantum-Particle-Swarm-Optimization-Based-Neural-Sharma-Kaushik/af2936752600a75a3579b37013bb1db3220bd078?p2df</x:v>
+      </x:c>
+      <x:c r="F92" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="2" t="str">
+        <x:v>Quantum Dilated Convolutional Neural Networks</x:v>
+      </x:c>
+      <x:c r="B93" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C93" s="2" t="str">
+        <x:v>IEEE Access</x:v>
+      </x:c>
+      <x:c r="D93" s="2" t="str">
+        <x:v>Yixiong Chen</x:v>
+      </x:c>
+      <x:c r="E93" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9715107</x:v>
+      </x:c>
+      <x:c r="F93" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="2" t="str">
+        <x:v>Efficient Quantum Image Classification Using Single Qubit Encoding</x:v>
+      </x:c>
+      <x:c r="B94" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C94" s="2" t="str">
+        <x:v>IEEE Transactions on Neural Networks and Learning Systems</x:v>
+      </x:c>
+      <x:c r="D94" s="2" t="str">
+        <x:v>Philip Easom-McCaldin; Ahmed Bouridane; Ammar Belatreche; Richard Jiang; Somaya Al-Maadeed</x:v>
+      </x:c>
+      <x:c r="E94" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9798852</x:v>
+      </x:c>
+      <x:c r="F94" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="2" t="str">
+        <x:v>Quantum-behaved particle swarm optimization of convolutional neural network for fault diagnosis</x:v>
+      </x:c>
+      <x:c r="B95" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C95" s="2" t="str">
+        <x:v>Journal of Experimental &amp; Theoretical Artificial Intelligence</x:v>
+      </x:c>
+      <x:c r="D95" s="2" t="str">
+        <x:v>Jie Chen , QingShan Xu , Xiaofeng Xue , Yingchao Guo &amp; Runfeng Chen</x:v>
+      </x:c>
+      <x:c r="E95" s="2" t="str">
+        <x:v>https://www.tandfonline.com/doi/abs/10.1080/0952813X.2022.2120089</x:v>
+      </x:c>
+      <x:c r="F95" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="2" t="str">
+        <x:v>Case study on quantum convolutional neural network scalability</x:v>
+      </x:c>
+      <x:c r="B96" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C96" s="2" t="str">
+        <x:v>arxiv</x:v>
+      </x:c>
+      <x:c r="D96" s="2" t="str">
+        <x:v>Marina O. Lisnichenko, Stanislav I. Protasov</x:v>
+      </x:c>
+      <x:c r="E96" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2207.07160</x:v>
+      </x:c>
+      <x:c r="F96" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="2" t="str">
+        <x:v>Poster: Scalable Quantum Convolutional Neural Networks for Edge Computing</x:v>
+      </x:c>
+      <x:c r="B97" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C97" s="2" t="str">
+        <x:v>2022 IEEE/ACM 7th Symposium on Edge Computing (SEC)</x:v>
+      </x:c>
+      <x:c r="D97" s="2" t="str">
+        <x:v>Jindi Wu; Qun Li</x:v>
+      </x:c>
+      <x:c r="E97" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9996801</x:v>
+      </x:c>
+      <x:c r="F97" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="2" t="str">
+        <x:v>A QCNN Algorithm Deployed on A Quantum Computer</x:v>
+      </x:c>
+      <x:c r="B98" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C98" s="2" t="str">
+        <x:v>2022 International Conference on Computing, Communication, Perception and Quantum Technology (CCPQT)</x:v>
+      </x:c>
+      <x:c r="D98" s="2" t="str">
+        <x:v>Xinmiao Chen; Bo Jiang; Yongzheng Wu; Yongjin Ye</x:v>
+      </x:c>
+      <x:c r="E98" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9939255</x:v>
+      </x:c>
+      <x:c r="F98" s="2" t="str">
+        <x:v>QCNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="2" t="str">
+        <x:v>Malaria Parasite Detection Using a Quantum-Convolutional Network</x:v>
+      </x:c>
+      <x:c r="B99" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C99" s="2" t="str">
         <x:v>Computers, Materials &amp; Continua</x:v>
       </x:c>
-      <x:c r="D92" s="2" t="str">
+      <x:c r="D99" s="2" t="str">
         <x:v>Javaria Amin 1 , Muhammad Almas Anjum2 , Abida Sharif 3 , Mudassar Raza 4 , Seifedine Kadry 5 and Yunyoung Nam</x:v>
       </x:c>
-      <x:c r="E92" s="2" t="str">
+      <x:c r="E99" s="2" t="str">
         <x:v>https://cdn.techscience.cn/ueditor/files/cmc/TSP_CMC-70-3/TSP_CMC_19115/TSP_CMC_19115.pdf</x:v>
       </x:c>
-      <x:c r="F92" s="2" t="str">
+      <x:c r="F99" s="2" t="str">
         <x:v>QCNN</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rbad82195de5f4f2a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rd88cbe6c86aa4c7a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R7be2567526004289"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="Rc2d13d4d37b74f95"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R211d85e17b9645b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R14348eddc9ba4253"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="Rdf4e4067de014b2f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="Rdce2b575406b4606"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Raa92dcc3f90342db"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R0e01d1efb4d64f7d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R7a8c2b280ecc45db"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R8e0033399e2e402f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R05e272a8ec3a487e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R42763403cdeb4044"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R1850bd5dcf704370"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="Rc3bc8a51feae4dd6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R4bbe461b64f14b8a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rd328c1b9273744a5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="R6e71e6bb7ff24a6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R28a78f271a014def"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R3c589b76259c4918"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="Rf8ba205476be4771"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R886f8cc7c0524620"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R26aacac734db4883"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="Rb939bc57f5134fdd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R734d48f32bbc4360"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R94edee7bcec845ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R77f541c6312d448a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R8872784b514d4a9b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Rf3aeeb9c5a8c44e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rb9b7deab311f4ba0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Rfd00ecf71674449a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R6be8d2c79ff84fde"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R8e0192c4999c4fc1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dca54db3af24b00"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R515af30780354afd"/>
 </x:worksheet>
 </file>
</xml_diff>